<commit_message>
Corrida | SFE-GCP | 2026-06-17 11:57:21.559314
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GCP_out.xlsx
+++ b/indicadores/SFE-GCP_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="429">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Gasto público de capital de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Gasto público de capital</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -71,6 +71,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -104,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/04/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1797,9 +1803,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>18</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1810,7 +1820,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1824,12 +1834,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.348817924153933</v>
+        <v>0.340965548007651</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1840,7 +1850,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -1868,7 +1878,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1882,12 +1892,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.121673944211059</v>
+        <v>0.116257504928158</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1910,7 +1920,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1924,7 +1934,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1938,7 +1948,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1952,12 +1962,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0284999350409865</v>
+        <v>0.013317096042514</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1968,7 +1978,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1982,12 +1992,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.508288829557334</v>
+        <v>0.498294396888329</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2130,10 +2140,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2146,10 +2156,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2173,66 +2183,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>1.39402218241627</v>
@@ -2285,7 +2295,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2.75709226452968</v>
@@ -2342,7 +2352,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>3.73711865970763</v>
@@ -2399,7 +2409,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>4.92634794554772</v>
@@ -2456,7 +2466,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>7.44271643046245</v>
@@ -2513,7 +2523,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>9.69892698613944</v>
@@ -2570,7 +2580,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>12.7321280480598</v>
@@ -2627,7 +2637,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>12.7074432266719</v>
@@ -2684,7 +2694,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>12.4558988188411</v>
@@ -2741,7 +2751,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>24.5869970136159</v>
@@ -2798,7 +2808,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>18.6974634752037</v>
@@ -2855,7 +2865,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>34.9040988547461</v>
@@ -2912,7 +2922,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>1.42906796897519</v>
@@ -2971,7 +2981,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>4.80560038268174</v>
@@ -3030,7 +3040,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>14.4432949593984</v>
@@ -3089,7 +3099,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>12.4899536368845</v>
@@ -3148,7 +3158,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>10.2427978152174</v>
@@ -3207,7 +3217,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>15.6684781297455</v>
@@ -3266,7 +3276,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>15.9340366287493</v>
@@ -3325,7 +3335,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>17.1153322043926</v>
@@ -3384,7 +3394,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>18.6485924124908</v>
@@ -3443,7 +3453,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>16.2852763249291</v>
@@ -3502,7 +3512,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>21.6806679990464</v>
@@ -3561,7 +3571,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>73.8917854564712</v>
@@ -3620,7 +3630,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>4.97961685621495</v>
@@ -3679,7 +3689,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>9.53357234376939</v>
@@ -3738,7 +3748,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>6.85103393366196</v>
@@ -3797,7 +3807,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>31.8179031947798</v>
@@ -3856,7 +3866,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>23.7797275167105</v>
@@ -3915,7 +3925,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>21.9138999238512</v>
@@ -3974,7 +3984,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>34.3715601556187</v>
@@ -4033,7 +4043,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>30.2990457038337</v>
@@ -4092,7 +4102,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>11.9548361557808</v>
@@ -4151,7 +4161,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>52.0547311464282</v>
@@ -4210,7 +4220,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>25.5407309187858</v>
@@ -4269,7 +4279,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>156.843748168353</v>
@@ -4328,7 +4338,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>16.2709700046856</v>
@@ -4387,7 +4397,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>9.88270719172036</v>
@@ -4446,7 +4456,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>37.9622979322888</v>
@@ -4505,7 +4515,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>37.0577854053482</v>
@@ -4564,7 +4574,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>43.9338069549648</v>
@@ -4623,7 +4633,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>54.7949068168876</v>
@@ -4682,7 +4692,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>48.2366649013119</v>
@@ -4741,7 +4751,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>55.358897229092</v>
@@ -4800,7 +4810,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>57.7567021598736</v>
@@ -4859,7 +4869,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>48.8515005600626</v>
@@ -4918,7 +4928,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>48.8448196640727</v>
@@ -4977,7 +4987,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>148.614002924266</v>
@@ -5036,7 +5046,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>18.6287973131261</v>
@@ -5095,7 +5105,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>25.5500959896994</v>
@@ -5154,7 +5164,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>34.1729415136388</v>
@@ -5213,7 +5223,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>32.2693161806385</v>
@@ -5272,7 +5282,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>30.2766065562392</v>
@@ -5331,7 +5341,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>42.4175204505264</v>
@@ -5390,7 +5400,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>38.1153022925306</v>
@@ -5449,7 +5459,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>40.9932011121215</v>
@@ -5508,7 +5518,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>47.9167770462345</v>
@@ -5567,7 +5577,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>32.1988108923993</v>
@@ -5626,7 +5636,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>53.5691077964842</v>
@@ -5685,7 +5695,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>66.7328722082852</v>
@@ -5744,7 +5754,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>7.60240290090359</v>
@@ -5803,7 +5813,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>18.2322856648001</v>
@@ -5862,7 +5872,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>24.7237834185111</v>
@@ -5921,7 +5931,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>26.5870971551146</v>
@@ -5980,7 +5990,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>28.2503343119457</v>
@@ -6039,7 +6049,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>23.4700318152747</v>
@@ -6098,7 +6108,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>35.7209088891522</v>
@@ -6157,7 +6167,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>38.3691258037819</v>
@@ -6216,7 +6226,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>33.5783366321348</v>
@@ -6275,7 +6285,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>46.0654375141221</v>
@@ -6334,7 +6344,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>40.6752181450451</v>
@@ -6393,7 +6403,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>139.249671332198</v>
@@ -6452,7 +6462,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>5.51672671296333</v>
@@ -6511,7 +6521,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>20.13681829726</v>
@@ -6570,7 +6580,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>30.2254190987607</v>
@@ -6629,7 +6639,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>26.7704889145147</v>
@@ -6688,7 +6698,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>33.4030475544683</v>
@@ -6747,7 +6757,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>26.8197026808547</v>
@@ -6806,7 +6816,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>44.1807343175025</v>
@@ -6865,7 +6875,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>27.4891510298957</v>
@@ -6924,7 +6934,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>34.202909455134</v>
@@ -6983,7 +6993,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>29.1215908740769</v>
@@ -7042,7 +7052,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>27.2672770168318</v>
@@ -7101,7 +7111,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>86.9728000850237</v>
@@ -7160,7 +7170,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>5.04621213214713</v>
@@ -7219,7 +7229,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>24.9875740161643</v>
@@ -7278,7 +7288,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>21.9122264351167</v>
@@ -7337,7 +7347,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>31.3361947671118</v>
@@ -7396,7 +7406,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>30.2769502002678</v>
@@ -7455,7 +7465,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>37.2252499110406</v>
@@ -7514,7 +7524,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>39.474683875579</v>
@@ -7573,7 +7583,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>44.1792463761318</v>
@@ -7632,7 +7642,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>35.3728525434246</v>
@@ -7691,7 +7701,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>25.3275246756612</v>
@@ -7750,7 +7760,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>42.1803399348963</v>
@@ -7809,7 +7819,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>110.089814050712</v>
@@ -7868,7 +7878,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>16.050186872136</v>
@@ -7927,7 +7937,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>18.603763271456</v>
@@ -7986,7 +7996,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>41.5969432431773</v>
@@ -8045,7 +8055,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>44.1157278505252</v>
@@ -8104,7 +8114,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>47.7130673188269</v>
@@ -8163,7 +8173,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>47.3136003619063</v>
@@ -8222,7 +8232,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>37.3631855982954</v>
@@ -8281,7 +8291,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>44.8309018142418</v>
@@ -8340,7 +8350,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>36.8005366545632</v>
@@ -8399,7 +8409,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>43.286999780306</v>
@@ -8458,7 +8468,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>35.2620282740179</v>
@@ -8517,7 +8527,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>85.1830083660647</v>
@@ -8576,7 +8586,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>17.6232090132096</v>
@@ -8635,7 +8645,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>16.2077217740133</v>
@@ -8694,7 +8704,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>24.1768723626175</v>
@@ -8753,7 +8763,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>21.6984780049455</v>
@@ -8812,7 +8822,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>31.1380964349369</v>
@@ -8871,7 +8881,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>30.969209902566</v>
@@ -8930,7 +8940,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>24.0041473928639</v>
@@ -8989,7 +8999,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>25.6423069658713</v>
@@ -9048,7 +9058,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>20.3634035596736</v>
@@ -9107,7 +9117,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>29.0081145011142</v>
@@ -9166,7 +9176,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>15.1861649474063</v>
@@ -9225,7 +9235,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>35.5805846325709</v>
@@ -9284,7 +9294,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>14.0171244320855</v>
@@ -9343,7 +9353,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>9.20403709254357</v>
@@ -9402,7 +9412,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>21.4184421336236</v>
@@ -9461,7 +9471,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>22.6582323401784</v>
@@ -9520,7 +9530,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>36.1307883230935</v>
@@ -9579,7 +9589,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>27.3397140164161</v>
@@ -9638,7 +9648,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>32.2706457890602</v>
@@ -9697,7 +9707,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>42.0746474333015</v>
@@ -9756,7 +9766,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>31.0046518492686</v>
@@ -9815,7 +9825,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>32.5080777776387</v>
@@ -9874,7 +9884,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>29.5539756578903</v>
@@ -9933,7 +9943,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>69.4396936616276</v>
@@ -9992,7 +10002,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>11.4239072353939</v>
@@ -10051,7 +10061,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>21.7308442708473</v>
@@ -10110,7 +10120,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>21.8123453142682</v>
@@ -10169,7 +10179,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>31.0499960280195</v>
@@ -10228,7 +10238,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>35.6150238732795</v>
@@ -10287,7 +10297,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>37.6676904713544</v>
@@ -10346,7 +10356,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>44.1817798410892</v>
@@ -10405,7 +10415,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>34.4762038223218</v>
@@ -10464,7 +10474,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>39.8932931697955</v>
@@ -10523,7 +10533,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>45.1485563548239</v>
@@ -10582,7 +10592,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>32.7596591518248</v>
@@ -10641,7 +10651,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>74.133511205701</v>
@@ -10700,7 +10710,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>26.4990687423212</v>
@@ -10759,7 +10769,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>25.0547003698948</v>
@@ -10818,7 +10828,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>54.3485098820197</v>
@@ -10877,7 +10887,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>46.0979480321964</v>
@@ -10936,7 +10946,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>52.2309163973978</v>
@@ -10995,7 +11005,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>47.3891122772208</v>
@@ -11054,7 +11064,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>52.7941511619362</v>
@@ -11113,7 +11123,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>42.7764202929092</v>
@@ -11172,7 +11182,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>52.052884853038</v>
@@ -11231,7 +11241,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>34.5326629003485</v>
@@ -11290,7 +11300,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>34.2579107540629</v>
@@ -11349,7 +11359,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>82.6124076038672</v>
@@ -11408,7 +11418,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>14.5008380071841</v>
@@ -11467,7 +11477,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>22.6593306412905</v>
@@ -11526,7 +11536,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>41.4593515354365</v>
@@ -11585,7 +11595,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>33.3665726421673</v>
@@ -11644,7 +11654,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>40.2278165067397</v>
@@ -11703,7 +11713,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>46.8690281591544</v>
@@ -11762,7 +11772,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>49.5682994922159</v>
@@ -11821,7 +11831,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>49.7801877370408</v>
@@ -11880,7 +11890,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>51.8175842702705</v>
@@ -11939,7 +11949,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>45.785858315648</v>
@@ -11998,7 +12008,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>64.5146225548992</v>
@@ -12057,7 +12067,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>115.240181561984</v>
@@ -12116,7 +12126,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>30.8206541308402</v>
@@ -12175,7 +12185,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>38.5791315780648</v>
@@ -12234,7 +12244,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>59.5508787536734</v>
@@ -12293,7 +12303,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>57.2165141677281</v>
@@ -12352,7 +12362,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>71.5274029053333</v>
@@ -12411,7 +12421,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>78.2669505181378</v>
@@ -12470,7 +12480,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>78.1537737749763</v>
@@ -12529,7 +12539,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>77.5017823980335</v>
@@ -12588,7 +12598,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>81.2403094058747</v>
@@ -12647,7 +12657,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>68.5269170093408</v>
@@ -12706,7 +12716,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>69.1286131878851</v>
@@ -12765,7 +12775,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>139.99108661652</v>
@@ -12824,7 +12834,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>24.3716131941066</v>
@@ -12883,7 +12893,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>58.2738028491121</v>
@@ -12942,7 +12952,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>73.0458351765862</v>
@@ -13001,7 +13011,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>67.116073059968</v>
@@ -13060,7 +13070,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>69.1831169291432</v>
@@ -13119,7 +13129,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>62.0905521538386</v>
@@ -13178,7 +13188,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>87.4269588497515</v>
@@ -13237,7 +13247,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>58.6349379319826</v>
@@ -13296,7 +13306,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>71.2354309075568</v>
@@ -13355,7 +13365,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>59.9315358376184</v>
@@ -13414,7 +13424,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>49.4394958177431</v>
@@ -13473,7 +13483,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>148.229318203944</v>
@@ -13532,7 +13542,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>57.0921782682537</v>
@@ -13591,7 +13601,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>52.2219713287285</v>
@@ -13650,7 +13660,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>55.4356464223824</v>
@@ -13709,7 +13719,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>66.1303456056788</v>
@@ -13768,7 +13778,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>79.1679256532187</v>
@@ -13827,7 +13837,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>63.7736634301749</v>
@@ -13886,7 +13896,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>67.5317747701022</v>
@@ -13945,7 +13955,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>53.949638008479</v>
@@ -14004,7 +14014,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>58.3227598422308</v>
@@ -14063,7 +14073,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>38.7017252982525</v>
@@ -14122,7 +14132,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>37.72520745497</v>
@@ -14181,7 +14191,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>90.5234778890356</v>
@@ -14240,7 +14250,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>4.97944769608538</v>
@@ -14299,7 +14309,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>14.4432991681674</v>
@@ -14358,7 +14368,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>16.0823826769043</v>
@@ -14417,7 +14427,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>8.44051836148453</v>
@@ -14476,7 +14486,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>16.2491495796053</v>
@@ -14535,7 +14545,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>19.8548478218819</v>
@@ -14594,7 +14604,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>19.1232568359563</v>
@@ -14653,7 +14663,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>22.381041201887</v>
@@ -14712,7 +14722,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>27.7802619990541</v>
@@ -14771,7 +14781,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>28.1745518211763</v>
@@ -14830,7 +14840,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>30.7715987166223</v>
@@ -14889,7 +14899,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>104.373822834149</v>
@@ -14948,7 +14958,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>11.1551602130825</v>
@@ -15007,7 +15017,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>14.0773109141039</v>
@@ -15066,7 +15076,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>32.1157775487792</v>
@@ -15125,7 +15135,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>29.4417790740693</v>
@@ -15184,7 +15194,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>28.4239868100221</v>
@@ -15243,7 +15253,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>37.2144019466941</v>
@@ -15302,7 +15312,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>36.1887693950945</v>
@@ -15361,7 +15371,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>42.0463772199899</v>
@@ -15420,7 +15430,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>55.8624939257297</v>
@@ -15479,7 +15489,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>36.5005165696192</v>
@@ -15538,7 +15548,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>49.6061622288209</v>
@@ -15597,7 +15607,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>71.7094554412269</v>
@@ -15656,7 +15666,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>13.7887985935928</v>
@@ -15715,7 +15725,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>30.8252990085616</v>
@@ -15774,7 +15784,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>42.6837271455702</v>
@@ -15833,7 +15843,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>35.7092497048696</v>
@@ -15892,7 +15902,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>46.4514286552399</v>
@@ -15951,7 +15961,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>50.2036154530052</v>
@@ -16010,7 +16020,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>56.0226857741961</v>
@@ -16069,7 +16079,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>31.849226124375</v>
@@ -16128,7 +16138,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>50.7888557204319</v>
@@ -16187,7 +16197,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>41.519703694875</v>
@@ -16246,7 +16256,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>56.5753622362345</v>
@@ -16305,7 +16315,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>61.3348928427774</v>
@@ -16364,7 +16374,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>56.47983884582</v>
@@ -16423,7 +16433,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>26.8299882735729</v>
@@ -16482,7 +16492,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>55.826342103127</v>
@@ -16541,7 +16551,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>41.6576321235815</v>
@@ -16600,7 +16610,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>27.2999244030375</v>
@@ -16659,7 +16669,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>35.8278582335663</v>
@@ -16718,7 +16728,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>27.9692950055222</v>
@@ -16777,7 +16787,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>36.6105688856868</v>
@@ -16836,7 +16846,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>22.9722899975935</v>
@@ -16895,7 +16905,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>28.3877741404975</v>
@@ -16954,7 +16964,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>18.1296841583603</v>
@@ -17013,7 +17023,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>51.7596720179838</v>
@@ -17072,7 +17082,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>4.35304910726263</v>
@@ -17131,7 +17141,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>10.106050728854</v>
@@ -17190,7 +17200,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>37.5606005098356</v>
@@ -17249,7 +17259,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>27.063505614413</v>
@@ -17308,7 +17318,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>35.2503980982722</v>
@@ -17367,7 +17377,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>25.4193997833155</v>
@@ -17426,7 +17436,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>53.3545707863581</v>
@@ -17485,7 +17495,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>52.0620631535281</v>
@@ -17544,7 +17554,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>50.1578338769608</v>
@@ -17603,7 +17613,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>50.2919945222037</v>
@@ -17662,7 +17672,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>54.2354457640755</v>
@@ -17721,7 +17731,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>93.9256725662913</v>
@@ -17780,7 +17790,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>46.6050051284197</v>
@@ -17839,7 +17849,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>42.5221215966777</v>
@@ -17898,7 +17908,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>52.6085746409758</v>
@@ -17957,7 +17967,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>47.3534126128695</v>
@@ -18016,7 +18026,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>61.0406660669693</v>
@@ -18075,7 +18085,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>53.6586212380322</v>
@@ -18134,7 +18144,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>61.040021635903</v>
@@ -18193,7 +18203,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>77.1375553072599</v>
@@ -18252,7 +18262,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>65.0303412528327</v>
@@ -18311,7 +18321,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>44.9902395286546</v>
@@ -18370,7 +18380,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>51.1994549013127</v>
@@ -18429,7 +18439,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>56.5426945967978</v>
@@ -18488,7 +18498,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B278" s="2"/>
       <c r="C278" s="3" t="n">
@@ -18521,7 +18531,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B279" s="2"/>
       <c r="C279" s="3" t="n">
@@ -18554,7 +18564,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B280" s="2"/>
       <c r="C280" s="3" t="n">
@@ -18587,7 +18597,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B281" s="2"/>
       <c r="C281" s="3" t="n">
@@ -18620,7 +18630,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B282" s="2"/>
       <c r="C282" s="3" t="n">
@@ -18653,7 +18663,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B283" s="2"/>
       <c r="C283" s="3" t="n">
@@ -18686,7 +18696,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B284" s="2"/>
       <c r="C284" s="3" t="n">
@@ -18719,7 +18729,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B285" s="2"/>
       <c r="C285" s="3" t="n">
@@ -18752,7 +18762,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B286" s="2"/>
       <c r="C286" s="3" t="n">
@@ -18785,7 +18795,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B287" s="2"/>
       <c r="C287" s="3" t="n">
@@ -18818,7 +18828,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B288" s="2"/>
       <c r="C288" s="3" t="n">
@@ -18851,7 +18861,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B289" s="2"/>
       <c r="C289" s="3" t="n">
@@ -18884,7 +18894,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B290" s="2"/>
       <c r="C290" s="3"/>
@@ -18907,7 +18917,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B291" s="2"/>
       <c r="C291" s="3"/>
@@ -18930,7 +18940,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B292" s="2"/>
       <c r="C292" s="3"/>
@@ -18953,7 +18963,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B293" s="2"/>
       <c r="C293" s="3"/>
@@ -18976,7 +18986,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B294" s="2"/>
       <c r="C294" s="3"/>
@@ -18999,7 +19009,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B295" s="2"/>
       <c r="C295" s="3"/>
@@ -19022,7 +19032,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B296" s="2"/>
       <c r="C296" s="3"/>
@@ -19045,7 +19055,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B297" s="2"/>
       <c r="C297" s="3"/>
@@ -19068,7 +19078,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B298" s="2"/>
       <c r="C298" s="3"/>
@@ -19091,7 +19101,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B299" s="2"/>
       <c r="C299" s="3"/>
@@ -19114,7 +19124,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B300" s="2"/>
       <c r="C300" s="3"/>
@@ -19137,7 +19147,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B301" s="2"/>
       <c r="C301" s="3"/>
@@ -19160,7 +19170,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B302" s="2"/>
       <c r="C302" s="3"/>
@@ -19183,7 +19193,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B303" s="2"/>
       <c r="C303" s="3"/>
@@ -19206,7 +19216,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B304" s="2"/>
       <c r="C304" s="3"/>
@@ -19229,7 +19239,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B305" s="2"/>
       <c r="C305" s="3"/>
@@ -19252,7 +19262,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B306" s="2"/>
       <c r="C306" s="3"/>
@@ -19275,7 +19285,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B307" s="2"/>
       <c r="C307" s="3"/>
@@ -19298,7 +19308,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B308" s="2"/>
       <c r="C308" s="3"/>
@@ -19321,7 +19331,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B309" s="2"/>
       <c r="C309" s="3"/>
@@ -19344,7 +19354,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B310" s="2"/>
       <c r="C310" s="3"/>
@@ -19367,7 +19377,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B311" s="2"/>
       <c r="C311" s="3"/>
@@ -19390,7 +19400,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B312" s="2"/>
       <c r="C312" s="3"/>
@@ -19413,7 +19423,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B313" s="2"/>
       <c r="C313" s="3"/>
@@ -19436,7 +19446,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B314" s="2"/>
       <c r="C314" s="3"/>
@@ -19459,7 +19469,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B315" s="2"/>
       <c r="C315" s="3"/>
@@ -19482,7 +19492,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B316" s="2"/>
       <c r="C316" s="3"/>
@@ -19505,7 +19515,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B317" s="2"/>
       <c r="C317" s="3"/>
@@ -19528,7 +19538,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B318" s="2"/>
       <c r="C318" s="3"/>
@@ -19551,7 +19561,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B319" s="2"/>
       <c r="C319" s="3"/>
@@ -19574,7 +19584,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B320" s="2"/>
       <c r="C320" s="3"/>
@@ -19597,7 +19607,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B321" s="2"/>
       <c r="C321" s="3"/>
@@ -19620,7 +19630,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B322" s="2"/>
       <c r="C322" s="3"/>
@@ -19643,7 +19653,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B323" s="2"/>
       <c r="C323" s="3"/>
@@ -19666,7 +19676,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B324" s="2"/>
       <c r="C324" s="3"/>
@@ -19689,7 +19699,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B325" s="2"/>
       <c r="C325" s="3"/>
@@ -19712,7 +19722,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B326" s="2"/>
       <c r="C326" s="3"/>
@@ -19735,7 +19745,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B327" s="2"/>
       <c r="C327" s="3"/>
@@ -19758,7 +19768,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B328" s="2"/>
       <c r="C328" s="3"/>
@@ -19781,7 +19791,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B329" s="2"/>
       <c r="C329" s="3"/>
@@ -19804,7 +19814,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B330" s="2"/>
       <c r="C330" s="3"/>
@@ -19827,7 +19837,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B331" s="2"/>
       <c r="C331" s="3"/>
@@ -19850,7 +19860,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B332" s="2"/>
       <c r="C332" s="3"/>
@@ -19873,7 +19883,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B333" s="2"/>
       <c r="C333" s="3"/>
@@ -19896,7 +19906,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B334" s="2"/>
       <c r="C334" s="3"/>
@@ -19919,7 +19929,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B335" s="2"/>
       <c r="C335" s="3"/>
@@ -19942,7 +19952,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B336" s="2"/>
       <c r="C336" s="3"/>
@@ -19965,7 +19975,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B337" s="2"/>
       <c r="C337" s="3"/>
@@ -19999,97 +20009,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
     </row>
   </sheetData>
@@ -20113,7 +20123,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -20123,160 +20133,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0356472236615481</v>
+        <v>-0.0386816194817888</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0126580732339567</v>
+        <v>-0.0141766223622492</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0078686073812575</v>
+        <v>0.00929283062835483</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.107919044906245</v>
+        <v>0.115707795619855</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.199332713382145</v>
+        <v>0.204103129999274</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.221130131271638</v>
+        <v>0.213665068506108</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.233450315729931</v>
+        <v>0.225260415661132</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.25020464569348</v>
+        <v>0.255564145193941</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.314965887866524</v>
+        <v>0.32337694249392</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.348817924153933</v>
+        <v>0.340965548007651</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.269543543278926</v>
+        <v>0.252171967230393</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.182501274755432</v>
+        <v>0.176131155100565</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.12612849800971</v>
+        <v>0.138063077957012</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0707201295464498</v>
+        <v>0.0856914116398495</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0339273685737758</v>
+        <v>0.0300174044056029</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.00902824607230004</v>
+        <v>-0.00349126518669689</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0221517343209681</v>
+        <v>-0.0192258707045528</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0388210334675303</v>
+        <v>-0.0270263915341158</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0474957690394953</v>
+        <v>-0.0483180549613834</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-GCP | 2026-07-02 10:03:17.738391
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GCP_out.xlsx
+++ b/indicadores/SFE-GCP_out.xlsx
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">24/06/2026</t>
+    <t xml:space="preserve">02/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -1863,7 +1863,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.343542124023917</v>
+        <v>0.343388096643954</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -1921,7 +1921,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.118021190978864</v>
+        <v>0.117915384916757</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -1991,7 +1991,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0472641003549275</v>
+        <v>0.0469373065921311</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2021,7 +2021,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.266627059856664</v>
+        <v>0.265514959014976</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -20322,7 +20322,7 @@
         <v>410</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0515625260575642</v>
+        <v>-0.0513185548851056</v>
       </c>
     </row>
     <row r="6">
@@ -20330,7 +20330,7 @@
         <v>411</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0284548742208908</v>
+        <v>-0.028006291761676</v>
       </c>
     </row>
     <row r="7">
@@ -20338,7 +20338,7 @@
         <v>412</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00094280163912975</v>
+        <v>-0.000875647071195644</v>
       </c>
     </row>
     <row r="8">
@@ -20346,7 +20346,7 @@
         <v>413</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0897577027799591</v>
+        <v>0.0895742849001757</v>
       </c>
     </row>
     <row r="9">
@@ -20354,7 +20354,7 @@
         <v>414</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.172614071266056</v>
+        <v>0.172675312579906</v>
       </c>
     </row>
     <row r="10">
@@ -20362,7 +20362,7 @@
         <v>415</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.207559773120918</v>
+        <v>0.207746407164522</v>
       </c>
     </row>
     <row r="11">
@@ -20370,7 +20370,7 @@
         <v>416</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.23698143090031</v>
+        <v>0.237166298874299</v>
       </c>
     </row>
     <row r="12">
@@ -20378,7 +20378,7 @@
         <v>417</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.265957890102137</v>
+        <v>0.26615681303233</v>
       </c>
     </row>
     <row r="13">
@@ -20386,7 +20386,7 @@
         <v>418</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.321327182036554</v>
+        <v>0.321351218158462</v>
       </c>
     </row>
     <row r="14">
@@ -20394,7 +20394,7 @@
         <v>419</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.343542124023917</v>
+        <v>0.343388096643954</v>
       </c>
     </row>
     <row r="15">
@@ -20402,7 +20402,7 @@
         <v>420</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.273594828647443</v>
+        <v>0.273549795237501</v>
       </c>
     </row>
     <row r="16">
@@ -20410,7 +20410,7 @@
         <v>421</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.198861776446498</v>
+        <v>0.198852387082516</v>
       </c>
     </row>
     <row r="17">
@@ -20418,7 +20418,7 @@
         <v>422</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.143150329953815</v>
+        <v>0.142863763737717</v>
       </c>
     </row>
     <row r="18">
@@ -20426,7 +20426,7 @@
         <v>423</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0852796903326362</v>
+        <v>0.0849631106428104</v>
       </c>
     </row>
     <row r="19">
@@ -20434,7 +20434,7 @@
         <v>424</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0443972141951368</v>
+        <v>0.0443908985989771</v>
       </c>
     </row>
     <row r="20">
@@ -20442,7 +20442,7 @@
         <v>425</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0137041928823041</v>
+        <v>0.0137553173187074</v>
       </c>
     </row>
     <row r="21">
@@ -20450,7 +20450,7 @@
         <v>426</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0284864185595939</v>
+        <v>-0.0286058568005052</v>
       </c>
     </row>
     <row r="22">
@@ -20458,7 +20458,7 @@
         <v>427</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.068676844149451</v>
+        <v>-0.0688134802104242</v>
       </c>
     </row>
     <row r="23">
@@ -20466,7 +20466,7 @@
         <v>428</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0906411625889264</v>
+        <v>-0.0907876726077931</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-GCP | 2026-08-03 11:28:22.354096
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GCP_out.xlsx
+++ b/indicadores/SFE-GCP_out.xlsx
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">02/07/2026</t>
+    <t xml:space="preserve">03/08/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">pcohan</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1863,7 +1863,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.343388096643954</v>
+        <v>0.353267144424631</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -1921,7 +1921,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.117915384916757</v>
+        <v>0.124797675329933</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -1991,7 +1991,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0469373065921311</v>
+        <v>0.0378427075187519</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2021,7 +2021,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.265514959014976</v>
+        <v>0.295146958951913</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -20322,7 +20322,7 @@
         <v>410</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0513185548851056</v>
+        <v>-0.0585371688179914</v>
       </c>
     </row>
     <row r="6">
@@ -20330,7 +20330,7 @@
         <v>411</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.028006291761676</v>
+        <v>-0.0280715389914451</v>
       </c>
     </row>
     <row r="7">
@@ -20338,7 +20338,7 @@
         <v>412</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.000875647071195644</v>
+        <v>-0.000793713088483848</v>
       </c>
     </row>
     <row r="8">
@@ -20346,7 +20346,7 @@
         <v>413</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0895742849001757</v>
+        <v>0.0816638877966777</v>
       </c>
     </row>
     <row r="9">
@@ -20354,7 +20354,7 @@
         <v>414</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.172675312579906</v>
+        <v>0.163554735234306</v>
       </c>
     </row>
     <row r="10">
@@ -20362,7 +20362,7 @@
         <v>415</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.207746407164522</v>
+        <v>0.202013619482575</v>
       </c>
     </row>
     <row r="11">
@@ -20370,7 +20370,7 @@
         <v>416</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.237166298874299</v>
+        <v>0.240497939647282</v>
       </c>
     </row>
     <row r="12">
@@ -20378,7 +20378,7 @@
         <v>417</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.26615681303233</v>
+        <v>0.281089232042257</v>
       </c>
     </row>
     <row r="13">
@@ -20386,7 +20386,7 @@
         <v>418</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.321351218158462</v>
+        <v>0.338937818460518</v>
       </c>
     </row>
     <row r="14">
@@ -20394,7 +20394,7 @@
         <v>419</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.343388096643954</v>
+        <v>0.353267144424631</v>
       </c>
     </row>
     <row r="15">
@@ -20402,7 +20402,7 @@
         <v>420</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.273549795237501</v>
+        <v>0.273944060439513</v>
       </c>
     </row>
     <row r="16">
@@ -20410,7 +20410,7 @@
         <v>421</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.198852387082516</v>
+        <v>0.198539356368145</v>
       </c>
     </row>
     <row r="17">
@@ -20418,7 +20418,7 @@
         <v>422</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.142863763737717</v>
+        <v>0.149725494347543</v>
       </c>
     </row>
     <row r="18">
@@ -20426,7 +20426,7 @@
         <v>423</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0849631106428104</v>
+        <v>0.0926559263282816</v>
       </c>
     </row>
     <row r="19">
@@ -20434,7 +20434,7 @@
         <v>424</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0443908985989771</v>
+        <v>0.0428058346844547</v>
       </c>
     </row>
     <row r="20">
@@ -20442,7 +20442,7 @@
         <v>425</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0137553173187074</v>
+        <v>0.00420804270246404</v>
       </c>
     </row>
     <row r="21">
@@ -20450,7 +20450,7 @@
         <v>426</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0286058568005052</v>
+        <v>-0.0319931053601684</v>
       </c>
     </row>
     <row r="22">
@@ -20458,7 +20458,7 @@
         <v>427</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0688134802104242</v>
+        <v>-0.0664265163243536</v>
       </c>
     </row>
     <row r="23">
@@ -20466,7 +20466,7 @@
         <v>428</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0907876726077931</v>
+        <v>-0.0897671634569797</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-GCP | 2026-09-04 10:15:29.784584
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GCP_out.xlsx
+++ b/indicadores/SFE-GCP_out.xlsx
@@ -110,13 +110,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">03/08/2026</t>
+    <t xml:space="preserve">04/09/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1863,7 +1863,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.353267144424631</v>
+        <v>0.354610202766022</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -1921,7 +1921,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.124797675329933</v>
+        <v>0.125748395905759</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -1991,7 +1991,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0378427075187519</v>
+        <v>0.0263939843785862</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2021,7 +2021,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.295146958951913</v>
+        <v>0.346229417330575</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -20322,7 +20322,7 @@
         <v>410</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0585371688179914</v>
+        <v>-0.0534294625020364</v>
       </c>
     </row>
     <row r="6">
@@ -20330,7 +20330,7 @@
         <v>411</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0280715389914451</v>
+        <v>-0.0219820824419169</v>
       </c>
     </row>
     <row r="7">
@@ -20338,7 +20338,7 @@
         <v>412</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.000793713088483848</v>
+        <v>0.000713520348111422</v>
       </c>
     </row>
     <row r="8">
@@ -20346,7 +20346,7 @@
         <v>413</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0816638877966777</v>
+        <v>0.087814500167353</v>
       </c>
     </row>
     <row r="9">
@@ -20354,7 +20354,7 @@
         <v>414</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.163554735234306</v>
+        <v>0.173580374816688</v>
       </c>
     </row>
     <row r="10">
@@ -20362,7 +20362,7 @@
         <v>415</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.202013619482575</v>
+        <v>0.201587662697805</v>
       </c>
     </row>
     <row r="11">
@@ -20370,7 +20370,7 @@
         <v>416</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.240497939647282</v>
+        <v>0.236735182409598</v>
       </c>
     </row>
     <row r="12">
@@ -20378,7 +20378,7 @@
         <v>417</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.281089232042257</v>
+        <v>0.285557200154999</v>
       </c>
     </row>
     <row r="13">
@@ -20386,7 +20386,7 @@
         <v>418</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.338937818460518</v>
+        <v>0.344775351915814</v>
       </c>
     </row>
     <row r="14">
@@ -20394,7 +20394,7 @@
         <v>419</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.353267144424631</v>
+        <v>0.354610202766022</v>
       </c>
     </row>
     <row r="15">
@@ -20402,7 +20402,7 @@
         <v>420</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.273944060439513</v>
+        <v>0.273303381325665</v>
       </c>
     </row>
     <row r="16">
@@ -20410,7 +20410,7 @@
         <v>421</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.198539356368145</v>
+        <v>0.197015465722577</v>
       </c>
     </row>
     <row r="17">
@@ -20418,7 +20418,7 @@
         <v>422</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.149725494347543</v>
+        <v>0.150334197453772</v>
       </c>
     </row>
     <row r="18">
@@ -20426,7 +20426,7 @@
         <v>423</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.0926559263282816</v>
+        <v>0.10028112541961</v>
       </c>
     </row>
     <row r="19">
@@ -20434,7 +20434,7 @@
         <v>424</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.0428058346844547</v>
+        <v>0.0472716421620287</v>
       </c>
     </row>
     <row r="20">
@@ -20442,7 +20442,7 @@
         <v>425</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.00420804270246404</v>
+        <v>-0.00628238052563761</v>
       </c>
     </row>
     <row r="21">
@@ -20450,7 +20450,7 @@
         <v>426</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0319931053601684</v>
+        <v>-0.0459732231879481</v>
       </c>
     </row>
     <row r="22">
@@ -20458,7 +20458,7 @@
         <v>427</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.0664265163243536</v>
+        <v>-0.0711877147011547</v>
       </c>
     </row>
     <row r="23">
@@ -20466,7 +20466,7 @@
         <v>428</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.0897671634569797</v>
+        <v>-0.0960725829046812</v>
       </c>
     </row>
     <row r="24">

</xml_diff>